<commit_message>
Refining GIS dashboard: integrated 13th parameter, standardized cluster naming, and optimized popup display
</commit_message>
<xml_diff>
--- a/clustering/Hasil_Distribusi_Zonasi_K4.xlsx
+++ b/clustering/Hasil_Distribusi_Zonasi_K4.xlsx
@@ -438,10 +438,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C2" t="n">
-        <v>35.09</v>
+        <v>35.73</v>
       </c>
     </row>
     <row r="3">
@@ -449,10 +449,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>160</v>
+        <v>215</v>
       </c>
       <c r="C3" t="n">
-        <v>25.52</v>
+        <v>34.29</v>
       </c>
     </row>
     <row r="4">
@@ -460,10 +460,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="C4" t="n">
-        <v>23.92</v>
+        <v>25.68</v>
       </c>
     </row>
     <row r="5">
@@ -471,10 +471,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>97</v>
+        <v>27</v>
       </c>
       <c r="C5" t="n">
-        <v>15.47</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="6">

</xml_diff>